<commit_message>
Expand repository: coordinate systems K-12 thread (101 total entries)
</commit_message>
<xml_diff>
--- a/Indigenous_Math_Data_Repository.xlsx
+++ b/Indigenous_Math_Data_Repository.xlsx
@@ -13,12 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource_Registry" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ojibwe_Numbers" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Story_Theme_Repository'!$A$1:$L$31</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Math_Domain_Crosswalk'!$A$1:$G$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'State_Mandates'!$A$1:$I$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Resource_Registry'!$A$1:$I$12</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -26,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,19 +33,14 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -60,11 +50,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002D6A4F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0095D5B2"/>
       </patternFill>
     </fill>
   </fills>
@@ -77,17 +62,8 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00B7B7B7"/>
-      </left>
-      <right style="thin">
-        <color rgb="00B7B7B7"/>
-      </right>
-      <top style="thin">
-        <color rgb="00B7B7B7"/>
-      </top>
       <bottom style="thin">
-        <color rgb="00B7B7B7"/>
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
@@ -96,13 +72,15 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -469,21 +447,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2408,8 +2386,565 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>K2-08</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>K-2</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Weaving a Grid</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Anishinaabe, Navajo, and many nations' weaving traditions</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Anishinaabe, Diné (Navajo), Multiple Nations</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Grid structure, rows and columns, position words (over/under, left/right), reference lines vs. objects</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Concrete</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Weave paper strips on a loom card. The warp strings go up-and-down and stay still — they are the frame. The weft strips go side-to-side and move. Point to the 3rd warp string from the left. Now point to where the 2nd weft strip crosses it. Can you describe any position on the loom using two numbers?</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>Cultural Practice + Math Research</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Warp = reference frame (axis analog), weft = positioned thread. Directly addresses the K-2 misconception of confusing axis labels with coordinate values. Many Indigenous nations practice weaving; frame as non-negotiable reference structure is universal to all loom types.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>K2-09</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>K-2</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Four Directions Orientation</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Pan-Indigenous directional framework</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Dakota, Lakota, Ojibwe, Multiple Nations</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Cardinal directions, spatial orientation, position and direction, reference points</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Concrete</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Stand in the center of the room. Face North (the direction of the cold wind). Turn to face East (where the sun rises). Your body is at the center — the directions are the reference frame around you. If you walk 3 steps North and 2 steps East, describe where you are.</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>Cultural Practice</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>The four directions (✜) are foundational to many Indigenous worldviews and appear in MN 2022 standards. This is a body-based coordinate system: the child IS the origin, the directions ARE the axes. Guugu Yimithirr Aboriginal Australians use absolute cardinal directions instead of relative left/right.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>35-09</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Bead Loom Coordinates</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Native American beadwork traditions, four-directions symmetry</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Ojibwe, Dakota, Shoshone-Bannock, Multiple Nations</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Ordered pairs, Cartesian coordinates (Quadrant I), plotting points, four-fold symmetry, reflection</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Representational</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Using the Virtual Bead Loom, place a red bead at (3, 5) and a blue bead at (5, 3). Are these the same point? Why does order matter in an ordered pair? Now create a design with four-fold symmetry — the four directions of the loom are like the four quadrants.</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>CSDT Research (Eglash)</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Ron Eglash's Virtual Bead Loom at csdt.org. Free tool. Students must TYPE coordinates, not click — forces distinction between grid reference and point. Four-directions = four-quadrant analog. Research shows statistically significant math gains. Beginner mode uses Quadrant I only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>35-10</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>3-5</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>Weaving Patterns as Coordinate Plots</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Navajo (Diné) textile design, Anishinaabe finger-weaving</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Diné (Navajo), Anishinaabe</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Coordinate plotting, pattern translation on a grid, color-coded position, systematic recording</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Representational</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Look at this woven pattern. On graph paper, color the squares to match the pattern. Now write the coordinates of every red square. Can you describe the pattern using only coordinate pairs? If you shift every point 2 units right, what happens to the design?</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>Cultural Practice + Math Research</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Bridges between physical weaving (concrete) and coordinate notation (representational). Students discover that a design IS a set of coordinate pairs — same data, different representation. Addresses translation/transformation concepts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>68-09</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Star Navigation Angles</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Yup'ik environmental navigation, MCC star navigation module</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Yup'ik</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Angles, angular measurement, protractor use, estimating angles, compass directions, degrees</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Representational</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>A Yup'ik navigator uses the position of the North Star above the horizon to determine latitude. If the star is 65° above the horizon, what is the navigator's approximate latitude? Measure the angle between two landmarks using a protractor — how does this help you navigate?</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>MCC Research (Lipka)</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Based on MCC 'Star Navigation: Explorations into Angles and Measurement' Grade 6 module. RCT evidence: rural treatment students outperformed urban treatment on spatial tasks. Uses environmental features (mountains, snowdrifts, star positions) as angle references.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>68-10</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>D/Lakota and Ojibwe Star Maps</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Dakota/Lakota and Ojibwe celestial knowledge, Native Skywatchers</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Dakota, Lakota, Ojibwe</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Coordinate systems, polar coordinates (intro), angular position, distance estimation, circular measurement</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Representational</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>The Ojibwe Giizhig Anung Masinaaigan (Sky Star Map) places Polaris at the center. Describe the position of Mooz (Moose constellation) using direction and angle from Polaris. How is this different from using (x, y) coordinates? When might a circular reference system work better than a grid?</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>Native Skywatchers (Annette Lee)</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Annette Lee (Lakota astrophysicist/artist) directs Native Skywatchers. Star maps organized with Polaris at center = polar coordinate system. Introduces students to the idea that DIFFERENT coordinate systems exist for different purposes. MN-specific: Dakota and Ojibwe nations. NASA-funded educator workshops available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>68-11</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Indigenous Cartography</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Multiple nations' mapping traditions</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>Multiple Nations</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Scale, proportion, coordinate systems, spatial reasoning, map reading, relative vs. absolute position</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Representational</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Compare a Western-style grid map of your school neighborhood with an Indigenous relational map that shows connections between important places. What information does each map capture? Create your own map that uses landmarks as reference points instead of a grid. What are the advantages and disadvantages?</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Cultural Practice + Academic Research</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Indigenous cartography often prioritizes relationships and routes over abstract grids. Students compare coordinate-based (Cartesian) vs. landmark-based (relational) position systems. Builds critical thinking about WHY we choose particular coordinate systems. Connects to Guugu Yimithirr absolute-direction navigation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>912-08</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Polynesian Wayfinding and Trigonometry</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Pacific Islander celestial navigation, star compass</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Hawaiian, Polynesian, Micronesian</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Trigonometric functions, polar coordinates, angular measurement, sine/cosine for position, vector navigation</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Polynesian navigators divided the horizon into 32 houses of 11.25° each. A navigator measures a star at 42° elevation. Using trigonometry, if the star's declination is known, calculate the navigator's latitude. Compare this polar-coordinate navigation system with Cartesian plotting on a nautical chart.</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Cultural Practice + Academic Research</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Pacific navigators used what we now call polar coordinates and trigonometric reasoning centuries before European formalization. The Hōkūle'a voyaging canoe project continues this tradition. 32-house star compass = 360° divided into precise angular sectors. Connects to unit circle in trig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>912-09</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Coordinate System Comparison</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Cross-cultural mathematical systems</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>Multiple Nations</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Cartesian vs. polar coordinates, transformation between systems, choosing appropriate coordinate systems, mathematical modeling</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>A Dakota star map uses Polaris as center with angular positions (polar). A Navajo weaving pattern uses a grid (Cartesian). Convert 3 star positions from polar (r, θ) to Cartesian (x, y) coordinates. When is each system more useful? Write a reflection: why might different cultures develop different coordinate systems?</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>Synthesis / Cross-Cultural</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Capstone entry for the coordinate systems thread. Students see that ALL coordinate systems are human inventions for describing position — no single system is 'more correct.' This is the IK-HABME principle: Indigenous knowledge systems ARE mathematics, expressed differently.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2420,797 +2955,544 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Math_Domain</t>
+          <t>Indigenous_Concept</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Indigenous_Concept</t>
+          <t>Standard_Math_Domain</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Nation(s)</t>
+          <t>Standard_Math_Topic</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Grade_Range</t>
+          <t>Grade_Band</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Standard_Curriculum_Connection</t>
+          <t>Digester_Tag</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>CRA_Phase_Best_Fit</t>
+          <t>Connection_Description</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Digester_Tag</t>
+          <t>Source</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Number &amp; Operations</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Ojibwe base-10 number system with classificatory endings</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Anishinaabe</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>NUM_INDIGENOUS_COUNTING</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Lakota large-number estimation (bison herds)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>NUM_ESTIMATION_CONTEXT</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Inter-tribal trading systems and equivalence</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>NUM_TRADING_EQUIV</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr"/>
+      <c r="G4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Body-proportional measuring (fathom, cubit, hand span)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>MEAS_BODY_UNITS</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Seasonal/environmental indicators for navigation</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>MEAS_SEASONAL_DATA</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Wild rice/fish harvest data (real data sets)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>MEAS_HARVEST_DATA</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Data sovereignty and critical data literacy</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>MEAS_DATA_SOVEREIGNTY</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr"/>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Beadwork coordinate systems</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>GEO_BEADWORK</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Weaving patterns (tessellation, iteration, symmetry)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>GEO_WEAVING</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr"/>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Basket weaving (3D geometry, algorithmic patterns)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>GEO_BASKET_3D</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Construction (smokehouse, fish rack)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>GEO_CONSTRUCTION</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Star navigation (angles, celestial positions)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>GEO_STAR_NAV</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Birch bark biting (fold symmetry)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>GEO_SYMMETRY_FOLD</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Iterative design processes in weaving/beadwork</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>ALG_ITERATIVE_DESIGN</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Proportional scaling (model to full-size artifacts)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>ALG_SCALING</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Growth patterns in creation stories</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>ALG_GROWTH_STORIES</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Treaty and demographic data analysis</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>STAT_TREATY_DATA</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Population estimation (bison, fish, waterfowl)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>STAT_POP_ESTIMATION</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Environmental and water quality data</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>STAT_ENVIRONMENTAL</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Language revitalization data</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>STAT_LANGUAGE_DATA</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr"/>
+      <c r="G21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Loom Warp/Weft as Reference Frame</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Geometry</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Coordinate Plane, Grid Structure</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>K-5</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Counting, place value, number words, classification</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Concrete</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>NUM_INDIGENOUS_COUNTING</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Number &amp; Operations</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Lakota large-number estimation (bison herds)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Lakota</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>3-8</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Place value, magnitude, estimation, scientific notation</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Representational</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>NUM_ESTIMATION_CONTEXT</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Number &amp; Operations</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Inter-tribal trading systems and equivalence</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Multiple nations</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>3-5</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Multiplication, division, equivalence, early ratio</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Representational</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>NUM_TRADING_EQUIV</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Measurement &amp; Data</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Body-proportional measuring (fathom, cubit, hand span)</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Yup'ik, Multiple</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>K-5</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Non-standard units, standard units, ratio, proportion</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Concrete</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>MEAS_BODY_UNITS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Measurement &amp; Data</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Seasonal/environmental indicators for navigation</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Dakota, Yup'ik</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>3-8</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Time, data over time, patterns, coordinate systems</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Representational</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>MEAS_SEASONAL_DATA</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Measurement &amp; Data</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Wild rice/fish harvest data (real data sets)</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Anishinaabe</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>3-12</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Data collection, central tendency, spread, sampling</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Representational</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>MEAS_HARVEST_DATA</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Measurement &amp; Data</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Data sovereignty and critical data literacy</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Dakota, Anishinaabe</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>3-12</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Data source analysis, bias, perspective, statistical ethics</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Abstract</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>MEAS_DATA_SOVEREIGNTY</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>GEO_LOOM_GRID</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Warp threads = fixed reference lines (axis analog); weft = positioned elements. Physical loom makes the distinction between reference frame and plotted point tactile and intuitive.</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Cultural Practice + Pedagogical Research</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Four Directions as Coordinate Axes</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Geometry</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Beadwork coordinate systems</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Ojibwe, Shoshone-Bannock</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>3-8</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Cartesian coordinates, symmetry, transformations</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Concrete</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>GEO_BEADWORK</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Coordinate Systems, Quadrants</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>K-8</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>GEO_FOUR_DIRECTIONS</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>The four cardinal directions provide an Indigenous analog to the four quadrants of the Cartesian plane. Used in Eglash's Virtual Bead Loom and deeply embedded in many nations' worldviews.</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>CSDT (Eglash) + Cultural Practice</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Polar Star Maps (Polaris-Centered)</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Geometry</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Weaving patterns (tessellation, iteration, symmetry)</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Dine (Navajo), Tlingit</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>3-12</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Tessellation, transformations, proportional reasoning</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Representational</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>GEO_WEAVING</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Polar Coordinates, Angle Measurement</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>6-12</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>GEO_POLAR_STARMAP</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>D/Lakota and Ojibwe star maps with Polaris at center = polar coordinate system. Position described by angle and distance from center, not x/y. Introduces students to alternative coordinate systems.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Native Skywatchers (Annette Lee)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Celestial Navigation Trigonometry</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Geometry</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Basket weaving (3D geometry, algorithmic patterns)</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Pomo, Tla'amin</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>5-12</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>3D geometry, surface area, volume, algorithms</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Representational</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>GEO_BASKET_3D</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Geometry</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Construction (smokehouse, fish rack)</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Yup'ik</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>3-8</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Properties of rectangles, prisms, perimeter, area, volume</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Concrete</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>GEO_CONSTRUCTION</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Geometry</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Star navigation (angles, celestial positions)</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Yup'ik, Dakota</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>5-12</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Angles, coordinate systems, vectors, trigonometry</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Abstract</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>GEO_STAR_NAV</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Geometry</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Birch bark biting (fold symmetry)</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Ojibwe</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>K-3</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Symmetry, congruence, folding, shapes</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Concrete</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>GEO_SYMMETRY_FOLD</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Algebra &amp; Functions</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Iterative design processes in weaving/beadwork</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Multiple nations</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>6-12</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Functions, iteration, transformation composition</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Representational</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>ALG_ITERATIVE_DESIGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Algebra &amp; Functions</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Proportional scaling (model to full-size artifacts)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Multiple nations</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>5-8</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Proportional reasoning, ratios, scale factors</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Representational</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>ALG_SCALING</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Algebra &amp; Functions</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Growth patterns in creation stories</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Multiple nations</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>6-12</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Exponential growth, function modeling</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Abstract</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>ALG_GROWTH_STORIES</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Statistics &amp; Probability</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Treaty and demographic data analysis</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Dakota, Ojibwe</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>6-12</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Percent change, sampling, inference, regression</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Abstract</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>STAT_TREATY_DATA</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Statistics &amp; Probability</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Population estimation (bison, fish, waterfowl)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Lakota, Multiple</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>6-12</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Sampling, estimation, inference, confidence</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Abstract</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>STAT_POP_ESTIMATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Statistics &amp; Probability</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Environmental and water quality data</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Multiple nations</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Trigonometric Functions, Unit Circle</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>9-12</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Regression, modeling, data analysis, prediction</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Abstract</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>STAT_ENVIRONMENTAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Statistics &amp; Probability</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Language revitalization data</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Ojibwe, Dakota</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>9-12</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Time series, regression, prediction, modeling</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Abstract</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>STAT_LANGUAGE_DATA</t>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>GEO_CELESTIAL_TRIG</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Polynesian/Micronesian star compass divides horizon into 32 houses (11.25° each). Latitude determination from star elevation uses trigonometric ratios. Navigators performed vector addition mentally.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Polynesian Voyaging Society + Academic Research</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3223,17 +3505,6 @@
   </sheetPr>
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="35" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -3283,477 +3554,476 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Montana</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>1972 (const.), 2005 (funded)</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Constitutional</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>All subjects, all grades</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Yes (in standards)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Indian Education for All (IEFA)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Mature (20+ years)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>50%+ teachers underutilized resources; coaching essential; 400+ resources developed</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Hawaii</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Constitutional</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Constitutional</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>All subjects</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Limited</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Native Hawaiian Education</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Mature</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Constitutional mandate provides strongest legal backing</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Washington</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Legislative</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>All subjects, PK-12</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Not yet explicit in math</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Yes (all 29 tribes)</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Since Time Immemorial</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Active implementation</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>All 29 tribes endorsed; tribal sovereignty framing is powerful</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Minnesota</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>2007 (statute), 2022 (standards)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Legislative + Standards</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>All subjects, embedded</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Yes (benchmarks with ✜ symbol)</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Yes (11 nations)</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Indigenous Education for All</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Implementation by 2027-28</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Four-directions benchmarks across grade levels; MDE provides tribally endorsed resources</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Oregon</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Legislative</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>5 subject areas</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Limited</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Tribal History/Shared History</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>Active implementation</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Place-based, contemporary, developmentally appropriate required by law</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>South Dakota</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>2007</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Legislative</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>K-12 courses</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Advisory council</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Oceti Sakowin Essential Understandings</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Essential Understandings framework similar to Montana model</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>North Dakota</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Legislative</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>K-12</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Limited guidance</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Native American Essential Understandings</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>Early implementation</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Looser guidelines than Oregon; teacher discretion is wider</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Wisconsin</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Various</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Legislative</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Social studies focus</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Limited</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Act 31</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Social studies focus; math integration opportunity exists but not mandated</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Connecticut</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Legislative</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Coursework requirement</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Limited</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Native American Studies</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>Early implementation</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Newest mandate; still developing resources</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Alaska</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>N/A (federal + state)</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Program-based</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Supplemental math modules</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Yes (MCC modules)</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Yes (Yup'ik elders)</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Math in a Cultural Context</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>Research-based, proven</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Only Indigenous math program with RCT evidence; 9 modules available</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3764,18 +4034,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3826,524 +4095,615 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Math in a Cultural Context (MCC)</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Curriculum Modules</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Jerry Lipka / UAF + Yup'ik elders</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Yup'ik</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>K-8</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>All domains</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>RCT (highest)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>uaf.edu/mcc/</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>9 modules; 4-6 weeks each; can map directly to Digester themes</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Culturally Situated Design Tools (CSDT)</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Web Software</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Ron Eglash / RPI</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Multiple nations</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>3-12</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Geometry, Algebra</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Quasi-experimental</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>csdt.org</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Virtual Bead Loom and Navajo Rug Weaver can be linked as resources in outputs</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Dakota/Lakota Math Connections</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Framework</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Sitting Bull College</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Lakota, Dakota</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>K-12</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>All domains</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Peer-reviewed framework</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Frontiers in Education 2023</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Epistemological framework; guides HOW to integrate, not just WHAT</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>IK-HABME Framework</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Theoretical Framework</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Garcia-Olp et al.</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Multiple nations</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>K-12</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>All domains</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Peer-reviewed</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Academic publications</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Core principle: Indigenous Knowledge HAS ALWAYS BEEN math education</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Alliance of Indigenous Math Circles</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Program</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Dr. Tatiana Shubin / AIMC</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Multiple nations</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>3-12</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>All domains</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Program evaluation</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>aimath.org</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>After-school model; problem sets available for adaptation</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Montana IEFA Resources</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Curriculum Library</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Montana OPI</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Montana tribes</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>K-12</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Limited math</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>State evaluation</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>opi.mt.gov</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>400+ resources; Essential Understandings framework transferable to MN</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Washington Since Time Immemorial</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Curriculum</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>OSPI + 29 tribes</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Washington tribes</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>PK-12</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Limited math</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>State-endorsed</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>ospi.k12.wa.us</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>All 29 tribes endorsed; tribal sovereignty framing model</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Indigenous Math Network</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Resource Hub</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>UBC</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Multiple nations</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>K-12</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>All domains</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Practitioner resources</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>indigenous.mathnetwork.educ.ubc.ca</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Lesson plans and educator networks; good for PD resources</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>MN IEFA Resources</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Standards Support</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>MN Dept of Education</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Dakota, Anishinaabe</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>K-12</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Math (benchmarks)</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>State standard</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>education.mn.gov</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Official tribally endorsed resources; primary alignment target</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Navajo Weaving Math Lesson</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Lesson Plan</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>NIEA / Illuminative</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>Dine (Navajo)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>3-5</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Geometry</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Practitioner-created</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>illuminative.org</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Ready-to-use lesson plan; weaving + geometry</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Ojibwe Number System Resources</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Language/Math</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Various Ojibwe educators</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Anishinaabe</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>K-5</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Number &amp; Operations</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Cultural authority</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>ojibwe.net</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Number words, classificatory endings; directly usable in Digester</t>
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Virtual Bead Loom (CSDT)</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Interactive Tool</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>RCT (Eglash et al.)</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+      <c r="I13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Native Skywatchers Star Maps</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Curriculum + Star Maps</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr"/>
+      <c r="F14" s="3" t="inlineStr"/>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Expert-Created (Annette Lee)</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>MCC Star Navigation Module</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Curriculum Module</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>RCT (Lipka et al.)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Hōkūle'a Polynesian Voyaging Resources</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Educational Content</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Cultural Authority</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4354,14 +4714,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -4386,226 +4740,228 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>bezhig</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>beh-ZHIG</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>niizh</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>NEEZH</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="D3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>niswi</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>NIS-wee</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>niiwin</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>NEE-win</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>naanan</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>NAH-nahn</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="D6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>ingodaaswo</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>in-go-DAHS-wo</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Compound: ingod (one) + aaswi (more than five)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>niizhwaaso</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>NEEZH-wah-so</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>Compound: niizh (two) + aaswi</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>niswaaso</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>NIS-wah-so</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Compound: niswi (three) + aaswi</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>zhaangaso</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>ZHAHN-gah-so</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
+      <c r="D10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>midaaso</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>mi-DAH-so</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>Base unit for tens</t>
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Classificatory Endings</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr"/>
+      <c r="C12" s="4" t="inlineStr"/>
+      <c r="D12" s="4" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>-gon / -gwan</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Counting days</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>e.g., niizho-gon = two days</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr"/>
+    </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Classificatory Endings</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>-gon / -gwan</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Counting days</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>e.g., niizho-gon = two days</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>-sag</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Counting wooden containers</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>e.g., niizh-sag = two barrels</t>
         </is>
       </c>
+      <c r="D14" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A14:D14"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>